<commit_message>
Deploying to main from @ open-resource-discovery/specification@f6f9521b72c1f68de3d417ba79b6456204ae0d7f 🚀
</commit_message>
<xml_diff>
--- a/specification/pr-229/spec-v1/interfaces/Document.xlsx
+++ b/specification/pr-229/spec-v1/interfaces/Document.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1495" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1498" uniqueCount="217">
   <si>
     <t>Entity Name</t>
   </si>
@@ -401,6 +401,9 @@
   </si>
   <si>
     <t>Capability</t>
+  </si>
+  <si>
+    <t>ontologyLayers</t>
   </si>
   <si>
     <t>relatedCapabilities</t>
@@ -1035,7 +1038,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D498"/>
+  <dimension ref="A1:D499"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5159,13 +5162,13 @@
         <v>129</v>
       </c>
       <c r="B295" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="C295" t="b">
         <v>0</v>
       </c>
       <c r="D295" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
@@ -5173,10 +5176,10 @@
         <v>129</v>
       </c>
       <c r="B296" t="s">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="C296" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D296" t="s">
         <v>6</v>
@@ -5187,10 +5190,10 @@
         <v>129</v>
       </c>
       <c r="B297" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C297" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D297" t="s">
         <v>6</v>
@@ -5201,7 +5204,7 @@
         <v>129</v>
       </c>
       <c r="B298" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C298" t="b">
         <v>0</v>
@@ -5215,7 +5218,7 @@
         <v>129</v>
       </c>
       <c r="B299" t="s">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="C299" t="b">
         <v>0</v>
@@ -5229,10 +5232,10 @@
         <v>129</v>
       </c>
       <c r="B300" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C300" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D300" t="s">
         <v>6</v>
@@ -5243,13 +5246,13 @@
         <v>129</v>
       </c>
       <c r="B301" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C301" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D301" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
@@ -5257,7 +5260,7 @@
         <v>129</v>
       </c>
       <c r="B302" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="C302" t="b">
         <v>0</v>
@@ -5271,13 +5274,13 @@
         <v>129</v>
       </c>
       <c r="B303" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C303" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D303" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
@@ -5285,10 +5288,10 @@
         <v>129</v>
       </c>
       <c r="B304" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C304" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D304" t="s">
         <v>6</v>
@@ -5299,10 +5302,10 @@
         <v>129</v>
       </c>
       <c r="B305" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C305" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D305" t="s">
         <v>6</v>
@@ -5313,7 +5316,7 @@
         <v>129</v>
       </c>
       <c r="B306" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C306" t="b">
         <v>1</v>
@@ -5327,13 +5330,13 @@
         <v>129</v>
       </c>
       <c r="B307" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C307" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D307" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
@@ -5341,13 +5344,13 @@
         <v>129</v>
       </c>
       <c r="B308" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C308" t="b">
         <v>0</v>
       </c>
       <c r="D308" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
@@ -5355,7 +5358,7 @@
         <v>129</v>
       </c>
       <c r="B309" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="C309" t="b">
         <v>0</v>
@@ -5369,7 +5372,7 @@
         <v>129</v>
       </c>
       <c r="B310" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="C310" t="b">
         <v>0</v>
@@ -5383,7 +5386,7 @@
         <v>129</v>
       </c>
       <c r="B311" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C311" t="b">
         <v>0</v>
@@ -5397,13 +5400,13 @@
         <v>129</v>
       </c>
       <c r="B312" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C312" t="b">
         <v>0</v>
       </c>
       <c r="D312" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
@@ -5411,13 +5414,13 @@
         <v>129</v>
       </c>
       <c r="B313" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C313" t="b">
         <v>0</v>
       </c>
       <c r="D313" t="s">
-        <v>63</v>
+        <v>9</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
@@ -5425,13 +5428,13 @@
         <v>129</v>
       </c>
       <c r="B314" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="C314" t="b">
         <v>0</v>
       </c>
       <c r="D314" t="s">
-        <v>9</v>
+        <v>63</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
@@ -5439,13 +5442,13 @@
         <v>129</v>
       </c>
       <c r="B315" t="s">
-        <v>55</v>
+        <v>92</v>
       </c>
       <c r="C315" t="b">
         <v>0</v>
       </c>
       <c r="D315" t="s">
-        <v>56</v>
+        <v>9</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
@@ -5453,13 +5456,13 @@
         <v>129</v>
       </c>
       <c r="B316" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C316" t="b">
         <v>0</v>
       </c>
       <c r="D316" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
@@ -5467,13 +5470,13 @@
         <v>129</v>
       </c>
       <c r="B317" t="s">
-        <v>130</v>
+        <v>57</v>
       </c>
       <c r="C317" t="b">
         <v>0</v>
       </c>
       <c r="D317" t="s">
-        <v>131</v>
+        <v>58</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
@@ -5481,13 +5484,13 @@
         <v>129</v>
       </c>
       <c r="B318" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C318" t="b">
         <v>0</v>
       </c>
       <c r="D318" t="s">
-        <v>9</v>
+        <v>132</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
@@ -5495,13 +5498,13 @@
         <v>129</v>
       </c>
       <c r="B319" t="s">
-        <v>94</v>
+        <v>123</v>
       </c>
       <c r="C319" t="b">
         <v>0</v>
       </c>
       <c r="D319" t="s">
-        <v>132</v>
+        <v>9</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
@@ -5509,13 +5512,13 @@
         <v>129</v>
       </c>
       <c r="B320" t="s">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="C320" t="b">
         <v>0</v>
       </c>
       <c r="D320" t="s">
-        <v>20</v>
+        <v>133</v>
       </c>
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
@@ -5523,13 +5526,13 @@
         <v>129</v>
       </c>
       <c r="B321" t="s">
-        <v>83</v>
+        <v>19</v>
       </c>
       <c r="C321" t="b">
         <v>0</v>
       </c>
       <c r="D321" t="s">
-        <v>84</v>
+        <v>20</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
@@ -5537,13 +5540,13 @@
         <v>129</v>
       </c>
       <c r="B322" t="s">
-        <v>27</v>
+        <v>83</v>
       </c>
       <c r="C322" t="b">
         <v>0</v>
       </c>
       <c r="D322" t="s">
-        <v>9</v>
+        <v>84</v>
       </c>
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
@@ -5551,7 +5554,7 @@
         <v>129</v>
       </c>
       <c r="B323" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C323" t="b">
         <v>0</v>
@@ -5565,7 +5568,7 @@
         <v>129</v>
       </c>
       <c r="B324" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C324" t="b">
         <v>0</v>
@@ -5579,7 +5582,7 @@
         <v>129</v>
       </c>
       <c r="B325" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C325" t="b">
         <v>0</v>
@@ -5593,13 +5596,13 @@
         <v>129</v>
       </c>
       <c r="B326" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C326" t="b">
         <v>0</v>
       </c>
       <c r="D326" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
@@ -5607,13 +5610,13 @@
         <v>129</v>
       </c>
       <c r="B327" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C327" t="b">
         <v>0</v>
       </c>
       <c r="D327" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
@@ -5621,13 +5624,13 @@
         <v>129</v>
       </c>
       <c r="B328" t="s">
-        <v>16</v>
+        <v>34</v>
       </c>
       <c r="C328" t="b">
         <v>0</v>
       </c>
       <c r="D328" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.25">
@@ -5635,38 +5638,38 @@
         <v>129</v>
       </c>
       <c r="B329" t="s">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="C329" t="b">
         <v>0</v>
       </c>
       <c r="D329" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B330" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C330" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D330" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B331" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="C331" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D331" t="s">
         <v>6</v>
@@ -5674,13 +5677,13 @@
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B332" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="C332" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D332" t="s">
         <v>6</v>
@@ -5688,10 +5691,10 @@
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B333" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C333" t="b">
         <v>1</v>
@@ -5702,38 +5705,38 @@
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B334" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C334" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D334" t="s">
-        <v>101</v>
+        <v>6</v>
       </c>
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B335" t="s">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="C335" t="b">
         <v>0</v>
       </c>
       <c r="D335" t="s">
-        <v>6</v>
+        <v>101</v>
       </c>
     </row>
     <row r="336" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B336" t="s">
-        <v>118</v>
+        <v>38</v>
       </c>
       <c r="C336" t="b">
         <v>0</v>
@@ -5747,10 +5750,10 @@
         <v>134</v>
       </c>
       <c r="B337" t="s">
-        <v>5</v>
+        <v>118</v>
       </c>
       <c r="C337" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D337" t="s">
         <v>6</v>
@@ -5758,13 +5761,13 @@
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B338" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C338" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D338" t="s">
         <v>6</v>
@@ -5772,41 +5775,41 @@
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B339" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C339" t="b">
         <v>0</v>
       </c>
       <c r="D339" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B340" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C340" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D340" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B341" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C341" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D341" t="s">
         <v>6</v>
@@ -5814,10 +5817,10 @@
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B342" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C342" t="b">
         <v>0</v>
@@ -5828,13 +5831,13 @@
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B343" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C343" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D343" t="s">
         <v>6</v>
@@ -5842,41 +5845,41 @@
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B344" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C344" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D344" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B345" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C345" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D345" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B346" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C346" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D346" t="s">
         <v>6</v>
@@ -5884,13 +5887,13 @@
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B347" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C347" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D347" t="s">
         <v>6</v>
@@ -5898,10 +5901,10 @@
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B348" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C348" t="b">
         <v>1</v>
@@ -5912,13 +5915,13 @@
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B349" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="C349" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D349" t="s">
         <v>6</v>
@@ -5926,136 +5929,136 @@
     </row>
     <row r="350" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A350" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B350" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C350" t="b">
         <v>0</v>
       </c>
       <c r="D350" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B351" t="s">
-        <v>135</v>
+        <v>61</v>
       </c>
       <c r="C351" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D351" t="s">
-        <v>51</v>
+        <v>9</v>
       </c>
     </row>
     <row r="352" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A352" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B352" t="s">
         <v>136</v>
       </c>
       <c r="C352" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D352" t="s">
-        <v>137</v>
+        <v>51</v>
       </c>
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B353" t="s">
+        <v>137</v>
+      </c>
+      <c r="C353" t="b">
+        <v>0</v>
+      </c>
+      <c r="D353" t="s">
         <v>138</v>
-      </c>
-      <c r="C353" t="b">
-        <v>0</v>
-      </c>
-      <c r="D353" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A354" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B354" t="s">
-        <v>19</v>
+        <v>139</v>
       </c>
       <c r="C354" t="b">
         <v>0</v>
       </c>
       <c r="D354" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="355" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A355" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B355" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C355" t="b">
         <v>0</v>
       </c>
       <c r="D355" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="356" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A356" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B356" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C356" t="b">
         <v>0</v>
       </c>
       <c r="D356" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="357" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A357" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B357" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C357" t="b">
         <v>0</v>
       </c>
       <c r="D357" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="358" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A358" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="B358" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C358" t="b">
         <v>0</v>
       </c>
       <c r="D358" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="359" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A359" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B359" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C359" t="b">
         <v>0</v>
@@ -6066,27 +6069,27 @@
     </row>
     <row r="360" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A360" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B360" t="s">
-        <v>135</v>
+        <v>12</v>
       </c>
       <c r="C360" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D360" t="s">
-        <v>51</v>
+        <v>6</v>
       </c>
     </row>
     <row r="361" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A361" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B361" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C361" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D361" t="s">
         <v>51</v>
@@ -6094,7 +6097,7 @@
     </row>
     <row r="362" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A362" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B362" t="s">
         <v>141</v>
@@ -6103,88 +6106,88 @@
         <v>0</v>
       </c>
       <c r="D362" t="s">
-        <v>142</v>
+        <v>51</v>
       </c>
     </row>
     <row r="363" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A363" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B363" t="s">
+        <v>142</v>
+      </c>
+      <c r="C363" t="b">
+        <v>0</v>
+      </c>
+      <c r="D363" t="s">
         <v>143</v>
-      </c>
-      <c r="C363" t="b">
-        <v>0</v>
-      </c>
-      <c r="D363" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="364" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A364" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B364" t="s">
+        <v>144</v>
+      </c>
+      <c r="C364" t="b">
+        <v>0</v>
+      </c>
+      <c r="D364" t="s">
         <v>145</v>
-      </c>
-      <c r="C364" t="b">
-        <v>0</v>
-      </c>
-      <c r="D364" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="365" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A365" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B365" t="s">
+        <v>146</v>
+      </c>
+      <c r="C365" t="b">
+        <v>0</v>
+      </c>
+      <c r="D365" t="s">
         <v>147</v>
-      </c>
-      <c r="C365" t="b">
-        <v>0</v>
-      </c>
-      <c r="D365" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="366" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A366" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B366" t="s">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="C366" t="b">
         <v>0</v>
       </c>
       <c r="D366" t="s">
-        <v>33</v>
+        <v>149</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A367" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="B367" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C367" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D367" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="368" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A368" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B368" t="s">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="C368" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D368" t="s">
         <v>6</v>
@@ -6192,7 +6195,7 @@
     </row>
     <row r="369" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A369" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B369" t="s">
         <v>151</v>
@@ -6201,46 +6204,46 @@
         <v>0</v>
       </c>
       <c r="D369" t="s">
-        <v>152</v>
+        <v>6</v>
       </c>
     </row>
     <row r="370" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A370" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B370" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="C370" t="b">
         <v>0</v>
       </c>
       <c r="D370" t="s">
-        <v>33</v>
+        <v>153</v>
       </c>
     </row>
     <row r="371" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A371" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B371" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C371" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D371" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="372" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A372" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B372" t="s">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="C372" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D372" t="s">
         <v>6</v>
@@ -6248,7 +6251,7 @@
     </row>
     <row r="373" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A373" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B373" t="s">
         <v>151</v>
@@ -6257,57 +6260,57 @@
         <v>0</v>
       </c>
       <c r="D373" t="s">
-        <v>154</v>
+        <v>6</v>
       </c>
     </row>
     <row r="374" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A374" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B374" t="s">
+        <v>152</v>
+      </c>
+      <c r="C374" t="b">
+        <v>0</v>
+      </c>
+      <c r="D374" t="s">
         <v>155</v>
-      </c>
-      <c r="C374" t="b">
-        <v>0</v>
-      </c>
-      <c r="D374" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="375" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A375" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B375" t="s">
-        <v>32</v>
+        <v>156</v>
       </c>
       <c r="C375" t="b">
         <v>0</v>
       </c>
       <c r="D375" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="376" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A376" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B376" t="s">
-        <v>157</v>
+        <v>32</v>
       </c>
       <c r="C376" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D376" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="377" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A377" t="s">
+        <v>157</v>
+      </c>
+      <c r="B377" t="s">
         <v>158</v>
-      </c>
-      <c r="B377" t="s">
-        <v>159</v>
       </c>
       <c r="C377" t="b">
         <v>1</v>
@@ -6318,10 +6321,10 @@
     </row>
     <row r="378" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A378" t="s">
+        <v>159</v>
+      </c>
+      <c r="B378" t="s">
         <v>160</v>
-      </c>
-      <c r="B378" t="s">
-        <v>5</v>
       </c>
       <c r="C378" t="b">
         <v>1</v>
@@ -6332,13 +6335,13 @@
     </row>
     <row r="379" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B379" t="s">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="C379" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D379" t="s">
         <v>6</v>
@@ -6346,7 +6349,7 @@
     </row>
     <row r="380" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B380" t="s">
         <v>151</v>
@@ -6355,46 +6358,46 @@
         <v>0</v>
       </c>
       <c r="D380" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="381" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B381" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="C381" t="b">
         <v>0</v>
       </c>
       <c r="D381" t="s">
-        <v>33</v>
+        <v>162</v>
       </c>
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B382" t="s">
-        <v>163</v>
+        <v>32</v>
       </c>
       <c r="C382" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D382" t="s">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B383" t="s">
-        <v>54</v>
+        <v>164</v>
       </c>
       <c r="C383" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D383" t="s">
         <v>6</v>
@@ -6402,13 +6405,13 @@
     </row>
     <row r="384" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B384" t="s">
-        <v>165</v>
+        <v>54</v>
       </c>
       <c r="C384" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D384" t="s">
         <v>6</v>
@@ -6416,10 +6419,10 @@
     </row>
     <row r="385" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
+        <v>165</v>
+      </c>
+      <c r="B385" t="s">
         <v>166</v>
-      </c>
-      <c r="B385" t="s">
-        <v>5</v>
       </c>
       <c r="C385" t="b">
         <v>1</v>
@@ -6430,10 +6433,10 @@
     </row>
     <row r="386" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B386" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C386" t="b">
         <v>1</v>
@@ -6444,24 +6447,24 @@
     </row>
     <row r="387" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B387" t="s">
-        <v>167</v>
+        <v>10</v>
       </c>
       <c r="C387" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D387" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="388" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B388" t="s">
-        <v>31</v>
+        <v>168</v>
       </c>
       <c r="C388" t="b">
         <v>0</v>
@@ -6472,52 +6475,52 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B389" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C389" t="b">
         <v>0</v>
       </c>
       <c r="D389" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="390" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A390" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B390" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C390" t="b">
         <v>0</v>
       </c>
       <c r="D390" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="391" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A391" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B391" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="C391" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D391" t="s">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="392" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A392" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B392" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="C392" t="b">
         <v>1</v>
@@ -6528,10 +6531,10 @@
     </row>
     <row r="393" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A393" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B393" t="s">
-        <v>169</v>
+        <v>52</v>
       </c>
       <c r="C393" t="b">
         <v>1</v>
@@ -6542,13 +6545,13 @@
     </row>
     <row r="394" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A394" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B394" t="s">
-        <v>12</v>
+        <v>170</v>
       </c>
       <c r="C394" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D394" t="s">
         <v>6</v>
@@ -6556,10 +6559,10 @@
     </row>
     <row r="395" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A395" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B395" t="s">
-        <v>99</v>
+        <v>12</v>
       </c>
       <c r="C395" t="b">
         <v>0</v>
@@ -6570,13 +6573,13 @@
     </row>
     <row r="396" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A396" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B396" t="s">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="C396" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D396" t="s">
         <v>6</v>
@@ -6584,10 +6587,10 @@
     </row>
     <row r="397" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A397" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B397" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C397" t="b">
         <v>1</v>
@@ -6598,13 +6601,13 @@
     </row>
     <row r="398" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A398" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B398" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C398" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D398" t="s">
         <v>6</v>
@@ -6615,10 +6618,10 @@
         <v>171</v>
       </c>
       <c r="B399" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C399" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D399" t="s">
         <v>6</v>
@@ -6626,10 +6629,10 @@
     </row>
     <row r="400" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A400" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B400" t="s">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="C400" t="b">
         <v>1</v>
@@ -6640,13 +6643,13 @@
     </row>
     <row r="401" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B401" t="s">
-        <v>12</v>
+        <v>99</v>
       </c>
       <c r="C401" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D401" t="s">
         <v>6</v>
@@ -6654,13 +6657,13 @@
     </row>
     <row r="402" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B402" t="s">
-        <v>98</v>
+        <v>12</v>
       </c>
       <c r="C402" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D402" t="s">
         <v>6</v>
@@ -6671,7 +6674,7 @@
         <v>172</v>
       </c>
       <c r="B403" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C403" t="b">
         <v>1</v>
@@ -6682,13 +6685,13 @@
     </row>
     <row r="404" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B404" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="C404" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D404" t="s">
         <v>6</v>
@@ -6696,13 +6699,13 @@
     </row>
     <row r="405" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B405" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="C405" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D405" t="s">
         <v>6</v>
@@ -6713,7 +6716,7 @@
         <v>173</v>
       </c>
       <c r="B406" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C406" t="b">
         <v>1</v>
@@ -6724,13 +6727,13 @@
     </row>
     <row r="407" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B407" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="C407" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D407" t="s">
         <v>6</v>
@@ -6738,13 +6741,13 @@
     </row>
     <row r="408" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B408" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="C408" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D408" t="s">
         <v>6</v>
@@ -6755,7 +6758,7 @@
         <v>174</v>
       </c>
       <c r="B409" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C409" t="b">
         <v>1</v>
@@ -6766,13 +6769,13 @@
     </row>
     <row r="410" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B410" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="C410" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D410" t="s">
         <v>6</v>
@@ -6780,13 +6783,13 @@
     </row>
     <row r="411" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B411" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
       <c r="C411" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D411" t="s">
         <v>6</v>
@@ -6797,10 +6800,10 @@
         <v>175</v>
       </c>
       <c r="B412" t="s">
-        <v>176</v>
+        <v>99</v>
       </c>
       <c r="C412" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D412" t="s">
         <v>6</v>
@@ -6808,10 +6811,10 @@
     </row>
     <row r="413" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B413" t="s">
-        <v>7</v>
+        <v>177</v>
       </c>
       <c r="C413" t="b">
         <v>0</v>
@@ -6822,10 +6825,10 @@
     </row>
     <row r="414" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B414" t="s">
-        <v>177</v>
+        <v>7</v>
       </c>
       <c r="C414" t="b">
         <v>0</v>
@@ -6836,128 +6839,128 @@
     </row>
     <row r="415" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B415" t="s">
-        <v>8</v>
+        <v>178</v>
       </c>
       <c r="C415" t="b">
         <v>0</v>
       </c>
       <c r="D415" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="416" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B416" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C416" t="b">
         <v>0</v>
       </c>
       <c r="D416" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="417" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B417" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C417" t="b">
         <v>0</v>
       </c>
       <c r="D417" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="418" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B418" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C418" t="b">
         <v>0</v>
       </c>
       <c r="D418" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="419" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B419" t="s">
-        <v>163</v>
+        <v>31</v>
       </c>
       <c r="C419" t="b">
         <v>0</v>
       </c>
       <c r="D419" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="420" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B420" t="s">
-        <v>8</v>
+        <v>164</v>
       </c>
       <c r="C420" t="b">
         <v>0</v>
       </c>
       <c r="D420" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="421" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B421" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C421" t="b">
         <v>0</v>
       </c>
       <c r="D421" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="422" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B422" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C422" t="b">
         <v>0</v>
       </c>
       <c r="D422" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="423" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B423" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C423" t="b">
         <v>0</v>
       </c>
       <c r="D423" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="424" spans="1:4" x14ac:dyDescent="0.25">
@@ -6965,21 +6968,21 @@
         <v>179</v>
       </c>
       <c r="B424" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C424" t="b">
         <v>0</v>
       </c>
       <c r="D424" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="425" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B425" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C425" t="b">
         <v>0</v>
@@ -6990,58 +6993,58 @@
     </row>
     <row r="426" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B426" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C426" t="b">
         <v>0</v>
       </c>
       <c r="D426" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="427" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B427" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C427" t="b">
         <v>0</v>
       </c>
       <c r="D427" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="428" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B428" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C428" t="b">
         <v>0</v>
       </c>
       <c r="D428" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="429" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A429" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B429" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C429" t="b">
         <v>0</v>
       </c>
       <c r="D429" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="430" spans="1:4" x14ac:dyDescent="0.25">
@@ -7049,24 +7052,24 @@
         <v>180</v>
       </c>
       <c r="B430" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="C430" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D430" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="431" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A431" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B431" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="C431" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D431" t="s">
         <v>6</v>
@@ -7074,10 +7077,10 @@
     </row>
     <row r="432" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A432" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B432" t="s">
-        <v>181</v>
+        <v>117</v>
       </c>
       <c r="C432" t="b">
         <v>0</v>
@@ -7088,13 +7091,13 @@
     </row>
     <row r="433" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A433" t="s">
+        <v>181</v>
+      </c>
+      <c r="B433" t="s">
         <v>182</v>
       </c>
-      <c r="B433" t="s">
-        <v>97</v>
-      </c>
       <c r="C433" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D433" t="s">
         <v>6</v>
@@ -7102,13 +7105,13 @@
     </row>
     <row r="434" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A434" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B434" t="s">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="C434" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D434" t="s">
         <v>6</v>
@@ -7116,10 +7119,10 @@
     </row>
     <row r="435" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A435" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B435" t="s">
-        <v>181</v>
+        <v>117</v>
       </c>
       <c r="C435" t="b">
         <v>0</v>
@@ -7130,10 +7133,10 @@
     </row>
     <row r="436" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A436" t="s">
+        <v>183</v>
+      </c>
+      <c r="B436" t="s">
         <v>182</v>
-      </c>
-      <c r="B436" t="s">
-        <v>183</v>
       </c>
       <c r="C436" t="b">
         <v>0</v>
@@ -7144,13 +7147,13 @@
     </row>
     <row r="437" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A437" t="s">
+        <v>183</v>
+      </c>
+      <c r="B437" t="s">
         <v>184</v>
       </c>
-      <c r="B437" t="s">
-        <v>185</v>
-      </c>
       <c r="C437" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D437" t="s">
         <v>6</v>
@@ -7158,10 +7161,10 @@
     </row>
     <row r="438" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A438" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B438" t="s">
-        <v>10</v>
+        <v>186</v>
       </c>
       <c r="C438" t="b">
         <v>1</v>
@@ -7172,13 +7175,13 @@
     </row>
     <row r="439" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A439" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B439" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C439" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D439" t="s">
         <v>6</v>
@@ -7186,38 +7189,38 @@
     </row>
     <row r="440" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A440" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B440" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C440" t="b">
         <v>0</v>
       </c>
       <c r="D440" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="441" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A441" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B441" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C441" t="b">
         <v>0</v>
       </c>
       <c r="D441" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="442" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A442" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B442" t="s">
-        <v>186</v>
+        <v>8</v>
       </c>
       <c r="C442" t="b">
         <v>0</v>
@@ -7228,27 +7231,27 @@
     </row>
     <row r="443" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A443" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B443" t="s">
-        <v>38</v>
+        <v>187</v>
       </c>
       <c r="C443" t="b">
         <v>0</v>
       </c>
       <c r="D443" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="444" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A444" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B444" t="s">
-        <v>188</v>
+        <v>38</v>
       </c>
       <c r="C444" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D444" t="s">
         <v>6</v>
@@ -7256,10 +7259,10 @@
     </row>
     <row r="445" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A445" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B445" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C445" t="b">
         <v>1</v>
@@ -7270,10 +7273,10 @@
     </row>
     <row r="446" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A446" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B446" t="s">
-        <v>10</v>
+        <v>186</v>
       </c>
       <c r="C446" t="b">
         <v>1</v>
@@ -7284,13 +7287,13 @@
     </row>
     <row r="447" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A447" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B447" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C447" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D447" t="s">
         <v>6</v>
@@ -7298,38 +7301,38 @@
     </row>
     <row r="448" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A448" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B448" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="C448" t="b">
         <v>0</v>
       </c>
       <c r="D448" t="s">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="449" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A449" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B449" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C449" t="b">
         <v>0</v>
       </c>
       <c r="D449" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="450" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A450" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B450" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
       <c r="C450" t="b">
         <v>0</v>
@@ -7340,27 +7343,27 @@
     </row>
     <row r="451" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A451" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B451" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="C451" t="b">
         <v>0</v>
       </c>
       <c r="D451" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="452" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A452" t="s">
-        <v>84</v>
+        <v>188</v>
       </c>
       <c r="B452" t="s">
-        <v>189</v>
+        <v>38</v>
       </c>
       <c r="C452" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D452" t="s">
         <v>6</v>
@@ -7371,10 +7374,10 @@
         <v>84</v>
       </c>
       <c r="B453" t="s">
-        <v>12</v>
+        <v>190</v>
       </c>
       <c r="C453" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D453" t="s">
         <v>6</v>
@@ -7382,52 +7385,52 @@
     </row>
     <row r="454" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A454" t="s">
-        <v>190</v>
+        <v>84</v>
       </c>
       <c r="B454" t="s">
-        <v>191</v>
+        <v>12</v>
       </c>
       <c r="C454" t="b">
         <v>0</v>
       </c>
       <c r="D454" t="s">
-        <v>192</v>
+        <v>6</v>
       </c>
     </row>
     <row r="455" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B455" t="s">
+        <v>192</v>
+      </c>
+      <c r="C455" t="b">
+        <v>0</v>
+      </c>
+      <c r="D455" t="s">
         <v>193</v>
-      </c>
-      <c r="C455" t="b">
-        <v>1</v>
-      </c>
-      <c r="D455" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="456" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
+        <v>191</v>
+      </c>
+      <c r="B456" t="s">
+        <v>194</v>
+      </c>
+      <c r="C456" t="b">
+        <v>1</v>
+      </c>
+      <c r="D456" t="s">
         <v>195</v>
-      </c>
-      <c r="B456" t="s">
-        <v>5</v>
-      </c>
-      <c r="C456" t="b">
-        <v>1</v>
-      </c>
-      <c r="D456" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="457" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B457" t="s">
-        <v>196</v>
+        <v>5</v>
       </c>
       <c r="C457" t="b">
         <v>1</v>
@@ -7438,10 +7441,10 @@
     </row>
     <row r="458" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
+        <v>196</v>
+      </c>
+      <c r="B458" t="s">
         <v>197</v>
-      </c>
-      <c r="B458" t="s">
-        <v>5</v>
       </c>
       <c r="C458" t="b">
         <v>1</v>
@@ -7452,10 +7455,10 @@
     </row>
     <row r="459" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B459" t="s">
-        <v>196</v>
+        <v>5</v>
       </c>
       <c r="C459" t="b">
         <v>1</v>
@@ -7469,7 +7472,7 @@
         <v>198</v>
       </c>
       <c r="B460" t="s">
-        <v>97</v>
+        <v>197</v>
       </c>
       <c r="C460" t="b">
         <v>1</v>
@@ -7480,10 +7483,10 @@
     </row>
     <row r="461" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B461" t="s">
-        <v>199</v>
+        <v>97</v>
       </c>
       <c r="C461" t="b">
         <v>1</v>
@@ -7494,10 +7497,10 @@
     </row>
     <row r="462" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
+        <v>199</v>
+      </c>
+      <c r="B462" t="s">
         <v>200</v>
-      </c>
-      <c r="B462" t="s">
-        <v>97</v>
       </c>
       <c r="C462" t="b">
         <v>1</v>
@@ -7508,10 +7511,10 @@
     </row>
     <row r="463" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B463" t="s">
-        <v>201</v>
+        <v>97</v>
       </c>
       <c r="C463" t="b">
         <v>1</v>
@@ -7522,10 +7525,10 @@
     </row>
     <row r="464" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
+        <v>201</v>
+      </c>
+      <c r="B464" t="s">
         <v>202</v>
-      </c>
-      <c r="B464" t="s">
-        <v>5</v>
       </c>
       <c r="C464" t="b">
         <v>1</v>
@@ -7553,7 +7556,7 @@
         <v>204</v>
       </c>
       <c r="B466" t="s">
-        <v>205</v>
+        <v>5</v>
       </c>
       <c r="C466" t="b">
         <v>1</v>
@@ -7564,10 +7567,10 @@
     </row>
     <row r="467" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
+        <v>205</v>
+      </c>
+      <c r="B467" t="s">
         <v>206</v>
-      </c>
-      <c r="B467" t="s">
-        <v>5</v>
       </c>
       <c r="C467" t="b">
         <v>1</v>
@@ -7578,13 +7581,13 @@
     </row>
     <row r="468" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B468" t="s">
-        <v>207</v>
+        <v>5</v>
       </c>
       <c r="C468" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D468" t="s">
         <v>6</v>
@@ -7592,13 +7595,13 @@
     </row>
     <row r="469" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
+        <v>207</v>
+      </c>
+      <c r="B469" t="s">
         <v>208</v>
       </c>
-      <c r="B469" t="s">
-        <v>5</v>
-      </c>
       <c r="C469" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D469" t="s">
         <v>6</v>
@@ -7606,13 +7609,13 @@
     </row>
     <row r="470" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B470" t="s">
-        <v>207</v>
+        <v>5</v>
       </c>
       <c r="C470" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D470" t="s">
         <v>6</v>
@@ -7623,10 +7626,10 @@
         <v>209</v>
       </c>
       <c r="B471" t="s">
-        <v>5</v>
+        <v>208</v>
       </c>
       <c r="C471" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D471" t="s">
         <v>6</v>
@@ -7634,13 +7637,13 @@
     </row>
     <row r="472" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B472" t="s">
-        <v>207</v>
+        <v>5</v>
       </c>
       <c r="C472" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D472" t="s">
         <v>6</v>
@@ -7651,10 +7654,10 @@
         <v>210</v>
       </c>
       <c r="B473" t="s">
-        <v>5</v>
+        <v>208</v>
       </c>
       <c r="C473" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D473" t="s">
         <v>6</v>
@@ -7662,13 +7665,13 @@
     </row>
     <row r="474" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B474" t="s">
-        <v>207</v>
+        <v>5</v>
       </c>
       <c r="C474" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D474" t="s">
         <v>6</v>
@@ -7679,10 +7682,10 @@
         <v>211</v>
       </c>
       <c r="B475" t="s">
-        <v>5</v>
+        <v>208</v>
       </c>
       <c r="C475" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D475" t="s">
         <v>6</v>
@@ -7690,13 +7693,13 @@
     </row>
     <row r="476" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B476" t="s">
-        <v>207</v>
+        <v>5</v>
       </c>
       <c r="C476" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D476" t="s">
         <v>6</v>
@@ -7707,10 +7710,10 @@
         <v>212</v>
       </c>
       <c r="B477" t="s">
-        <v>5</v>
+        <v>208</v>
       </c>
       <c r="C477" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D477" t="s">
         <v>6</v>
@@ -7724,7 +7727,7 @@
         <v>5</v>
       </c>
       <c r="C478" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D478" t="s">
         <v>6</v>
@@ -7732,10 +7735,10 @@
     </row>
     <row r="479" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B479" t="s">
-        <v>188</v>
+        <v>5</v>
       </c>
       <c r="C479" t="b">
         <v>0</v>
@@ -7746,10 +7749,10 @@
     </row>
     <row r="480" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B480" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C480" t="b">
         <v>0</v>
@@ -7760,13 +7763,13 @@
     </row>
     <row r="481" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B481" t="s">
-        <v>214</v>
+        <v>186</v>
       </c>
       <c r="C481" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D481" t="s">
         <v>6</v>
@@ -7774,13 +7777,13 @@
     </row>
     <row r="482" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A482" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B482" t="s">
-        <v>12</v>
+        <v>215</v>
       </c>
       <c r="C482" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D482" t="s">
         <v>6</v>
@@ -7788,13 +7791,13 @@
     </row>
     <row r="483" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A483" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B483" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C483" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D483" t="s">
         <v>6</v>
@@ -7802,13 +7805,13 @@
     </row>
     <row r="484" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A484" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B484" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C484" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D484" t="s">
         <v>6</v>
@@ -7816,41 +7819,41 @@
     </row>
     <row r="485" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A485" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B485" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C485" t="b">
         <v>0</v>
       </c>
       <c r="D485" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="486" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A486" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B486" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C486" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D486" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="487" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A487" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B487" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C487" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D487" t="s">
         <v>6</v>
@@ -7858,13 +7861,13 @@
     </row>
     <row r="488" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A488" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B488" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C488" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D488" t="s">
         <v>6</v>
@@ -7872,10 +7875,10 @@
     </row>
     <row r="489" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A489" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B489" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C489" t="b">
         <v>1</v>
@@ -7886,41 +7889,41 @@
     </row>
     <row r="490" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A490" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B490" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C490" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D490" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="491" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A491" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B491" t="s">
-        <v>13</v>
+        <v>46</v>
       </c>
       <c r="C491" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D491" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="492" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A492" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B492" t="s">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C492" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D492" t="s">
         <v>6</v>
@@ -7928,13 +7931,13 @@
     </row>
     <row r="493" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A493" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B493" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C493" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D493" t="s">
         <v>6</v>
@@ -7942,10 +7945,10 @@
     </row>
     <row r="494" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A494" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B494" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="C494" t="b">
         <v>1</v>
@@ -7956,57 +7959,71 @@
     </row>
     <row r="495" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A495" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B495" t="s">
-        <v>19</v>
+        <v>52</v>
       </c>
       <c r="C495" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D495" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="496" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A496" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B496" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="C496" t="b">
         <v>0</v>
       </c>
       <c r="D496" t="s">
-        <v>9</v>
+        <v>20</v>
       </c>
     </row>
     <row r="497" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A497" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B497" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C497" t="b">
         <v>0</v>
       </c>
       <c r="D497" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
     </row>
     <row r="498" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A498" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B498" t="s">
+        <v>32</v>
+      </c>
+      <c r="C498" t="b">
+        <v>0</v>
+      </c>
+      <c r="D498" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="499" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A499" t="s">
+        <v>216</v>
+      </c>
+      <c r="B499" t="s">
         <v>34</v>
       </c>
-      <c r="C498" t="b">
-        <v>0</v>
-      </c>
-      <c r="D498" t="s">
+      <c r="C499" t="b">
+        <v>0</v>
+      </c>
+      <c r="D499" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>